<commit_message>
Update analisis part 1
</commit_message>
<xml_diff>
--- a/analisis/entropy_results.xlsx
+++ b/analisis/entropy_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,21 @@
           <t>overhead_relativo</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>\%_bpp_bit</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>\%_bpp_raw</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>real_impacto</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -519,6 +534,15 @@
       <c r="K2" t="n">
         <v>24.76568049758238</v>
       </c>
+      <c r="L2" t="n">
+        <v>91.01553000034743</v>
+      </c>
+      <c r="M2" t="n">
+        <v>8.984469999652571</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2.225065134515096</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -554,6 +578,15 @@
       <c r="K3" t="n">
         <v>23.89445407756255</v>
       </c>
+      <c r="L3" t="n">
+        <v>86.33299422017015</v>
+      </c>
+      <c r="M3" t="n">
+        <v>13.66700577982985</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3.265656419839263</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -589,6 +622,15 @@
       <c r="K4" t="n">
         <v>39.14353071179054</v>
       </c>
+      <c r="L4" t="n">
+        <v>79.29553209192525</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20.70446790807474</v>
+      </c>
+      <c r="N4" t="n">
+        <v>8.104459754310051</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -624,6 +666,15 @@
       <c r="K5" t="n">
         <v>32.46920826240704</v>
       </c>
+      <c r="L5" t="n">
+        <v>69.54482758620689</v>
+      </c>
+      <c r="M5" t="n">
+        <v>30.45517241379311</v>
+      </c>
+      <c r="N5" t="n">
+        <v>9.888553357709622</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -658,6 +709,15 @@
       </c>
       <c r="K6" t="n">
         <v>8.26408556799665</v>
+      </c>
+      <c r="L6" t="n">
+        <v>54.15872824523105</v>
+      </c>
+      <c r="M6" t="n">
+        <v>45.84127175476895</v>
+      </c>
+      <c r="N6" t="n">
+        <v>3.788361923271986</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Pipeline + analisis part
</commit_message>
<xml_diff>
--- a/analisis/entropy_results.xlsx
+++ b/analisis/entropy_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,62 +441,67 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>H_seq</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H_seq_cxt</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Bits_per_pixel_seq</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>H_bits</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>H_limit_total</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>H_limit_bits</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>H_limit_raw</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>bpp_final</t>
+          <t>H_bits_cxt</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>bpp_bits</t>
+          <t>Exp_bit_rate_only_bits_seq</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>bpp_raw</t>
+          <t>Exp_bit_rate</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>overhead_raw</t>
+          <t>Exp_bit_rate_bits</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>overhead_relativo</t>
+          <t>Exp_bit_rate_raw</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>\%_bpp_bit</t>
+          <t>bit_rate_final</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>\%_bpp_raw</t>
+          <t>bit_rate_offline</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>real_impacto</t>
+          <t>bit_rate_bits</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>bit_rate_raw</t>
         </is>
       </c>
     </row>
@@ -505,219 +510,140 @@
         <v>4</v>
       </c>
       <c r="B2" t="n">
-        <v>1.539776224154324</v>
+        <v>1.701959107500815</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3192749730364189</v>
+        <v>1.316332432149416</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1785281579465127</v>
+        <v>0.9371797366220725</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1661505654286195</v>
+        <v>0.9371797366220725</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01237759251789317</v>
+        <v>0.8592444892531783</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1831166021986971</v>
+        <v>0.7224904408531194</v>
       </c>
       <c r="H2" t="n">
-        <v>0.166664546009772</v>
+        <v>1.114570489239136</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01645205618892508</v>
+        <v>1.050745632379464</v>
       </c>
       <c r="J2" t="n">
-        <v>0.004074463671031913</v>
+        <v>0.9371797366220722</v>
       </c>
       <c r="K2" t="n">
-        <v>24.76568049758238</v>
+        <v>0.1135658957573916</v>
       </c>
       <c r="L2" t="n">
-        <v>91.01553000034743</v>
+        <v>1.077275676913681</v>
       </c>
       <c r="M2" t="n">
-        <v>8.984469999652571</v>
+        <v>1.07656631718241</v>
       </c>
       <c r="N2" t="n">
-        <v>2.225065134515096</v>
+        <v>0.9378976231677525</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.1393780537459283</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>2.11699295093553</v>
+        <v>3.255536237665001</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4309861533484639</v>
+        <v>1.998343780748378</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2746833915496202</v>
+        <v>1.371365356298331</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2450878125179822</v>
+        <v>1.371365356298331</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02959557903163801</v>
+        <v>0.9982229216988844</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2845359578583062</v>
+        <v>0.8665926624912178</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2456484120521173</v>
+        <v>1.579667578473899</v>
       </c>
       <c r="I3" t="n">
-        <v>0.03888754580618892</v>
+        <v>1.898349917041454</v>
       </c>
       <c r="J3" t="n">
-        <v>0.009291966774550915</v>
+        <v>1.37136535629833</v>
       </c>
       <c r="K3" t="n">
-        <v>23.89445407756255</v>
+        <v>0.5269845607431237</v>
       </c>
       <c r="L3" t="n">
-        <v>86.33299422017015</v>
+        <v>2.05010370012215</v>
       </c>
       <c r="M3" t="n">
-        <v>13.66700577982985</v>
+        <v>2.049349806596091</v>
       </c>
       <c r="N3" t="n">
-        <v>3.265656419839263</v>
+        <v>1.372121208265472</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.6779824918566775</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>2.74410681245273</v>
+        <v>3.843323198207317</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6088708664016617</v>
+        <v>2.280076473250217</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4526124895109409</v>
+        <v>1.56483043180701</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3904721742068538</v>
+        <v>1.56483043180701</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06214031530408705</v>
+        <v>0.9862375052416633</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4931767864413681</v>
+        <v>0.8807946378512583</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3910671569625407</v>
+        <v>1.75216150833584</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1021096294788274</v>
+        <v>2.437648206554485</v>
       </c>
       <c r="J4" t="n">
-        <v>0.03996931417474031</v>
+        <v>1.564830431807011</v>
       </c>
       <c r="K4" t="n">
-        <v>39.14353071179054</v>
+        <v>0.8728177747474744</v>
       </c>
       <c r="L4" t="n">
-        <v>79.29553209192525</v>
+        <v>2.502392100977199</v>
       </c>
       <c r="M4" t="n">
-        <v>20.70446790807474</v>
+        <v>2.501619121539088</v>
       </c>
       <c r="N4" t="n">
-        <v>8.104459754310051</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>17</v>
-      </c>
-      <c r="B5" t="n">
-        <v>3.704062898962805</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.9527072479614129</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.8305984842982388</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.6408743544165647</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.189724129881674</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9224857491856677</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.6415411237785016</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.2809446254071661</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.09122049552549211</v>
-      </c>
-      <c r="K5" t="n">
-        <v>32.46920826240704</v>
-      </c>
-      <c r="L5" t="n">
-        <v>69.54482758620689</v>
-      </c>
-      <c r="M5" t="n">
-        <v>30.45517241379311</v>
-      </c>
-      <c r="N5" t="n">
-        <v>9.888553357709622</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B6" t="n">
-        <v>4.871331120463552</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1.723044400277364</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2.334884214382668</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1.313999423803977</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.020884790578692</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2.427619859527687</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1.31476804254886</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1.112851816978827</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.09196702640013577</v>
-      </c>
-      <c r="K6" t="n">
-        <v>8.26408556799665</v>
-      </c>
-      <c r="L6" t="n">
-        <v>54.15872824523105</v>
-      </c>
-      <c r="M6" t="n">
-        <v>45.84127175476895</v>
-      </c>
-      <c r="N6" t="n">
-        <v>3.788361923271986</v>
+        <v>1.565604641693811</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.9367874592833876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>